<commit_message>
version 40 - Combine VNPay payment gateway
</commit_message>
<xml_diff>
--- a/Documentation/Parameter_configuration/Parameter_Design.xlsx
+++ b/Documentation/Parameter_configuration/Parameter_Design.xlsx
@@ -106,6 +106,13 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
       <t xml:space="preserve">- </t>
     </r>
     <r>
@@ -270,6 +277,13 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
       <t xml:space="preserve">- </t>
     </r>
     <r>
@@ -450,7 +464,7 @@
         <charset val="134"/>
         <scheme val="minor"/>
       </rPr>
-      <t>TRUE</t>
+      <t>FALSE</t>
     </r>
     <r>
       <rPr>
@@ -472,7 +486,7 @@
         <charset val="134"/>
         <scheme val="minor"/>
       </rPr>
-      <t>None (Different origin)</t>
+      <t>lax (Same origin localhost)</t>
     </r>
   </si>
   <si>
@@ -480,6 +494,13 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
       <t xml:space="preserve">Server API is: </t>
     </r>
     <r>
@@ -496,6 +517,13 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
       <t xml:space="preserve">Server API is: </t>
     </r>
     <r>
@@ -512,6 +540,13 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
       <t xml:space="preserve">Server API is: </t>
     </r>
     <r>
@@ -718,7 +753,7 @@
     <font>
       <b/>
       <sz val="11"/>
-      <color rgb="FF00B0F0"/>
+      <color theme="9" tint="-0.25"/>
       <name val="Calibri"/>
       <charset val="134"/>
       <scheme val="minor"/>
@@ -726,13 +761,13 @@
     <font>
       <b/>
       <sz val="11"/>
-      <color theme="9" tint="-0.25"/>
+      <color rgb="FF00B0F0"/>
       <name val="Calibri"/>
       <charset val="134"/>
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="37">
+  <fills count="36">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -748,12 +783,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="5" tint="0.6"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.4"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1097,7 +1126,7 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="2" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="2" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -1121,16 +1150,16 @@
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="7" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="8" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="8" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="9" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="13" fillId="6" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="7" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="7" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="8" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="17" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
@@ -1139,89 +1168,89 @@
     <xf numFmtId="0" fontId="18" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="19" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="23" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="22" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="23" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="23" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="22" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="23" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="23" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="22" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="23" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="23" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="22" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="23" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="23" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="22" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="23" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="23" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="36" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -1234,16 +1263,10 @@
     <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1252,10 +1275,10 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
@@ -1266,9 +1289,6 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1">
       <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -1867,170 +1887,170 @@
   </cols>
   <sheetData>
     <row r="1" spans="3:6">
-      <c r="C1" s="9"/>
-      <c r="D1" s="9"/>
-      <c r="E1" s="9"/>
-      <c r="F1" s="9"/>
+      <c r="C1" s="7"/>
+      <c r="D1" s="7"/>
+      <c r="E1" s="7"/>
+      <c r="F1" s="7"/>
     </row>
     <row r="2" spans="2:6">
-      <c r="B2" s="10" t="s">
+      <c r="B2" s="8" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="11" t="s">
+      <c r="C2" s="9" t="s">
         <v>1</v>
       </c>
-      <c r="D2" s="11" t="s">
+      <c r="D2" s="9" t="s">
         <v>2</v>
       </c>
-      <c r="E2" s="11" t="s">
+      <c r="E2" s="9" t="s">
         <v>3</v>
       </c>
-      <c r="F2" s="9"/>
+      <c r="F2" s="7"/>
     </row>
     <row r="3" spans="2:6">
-      <c r="B3" s="12" t="s">
+      <c r="B3" s="10" t="s">
         <v>4</v>
       </c>
-      <c r="C3" s="13" t="s">
+      <c r="C3" s="11" t="s">
         <v>5</v>
       </c>
-      <c r="D3" s="14" t="b">
+      <c r="D3" s="12" t="b">
         <v>1</v>
       </c>
-      <c r="E3" s="14" t="s">
+      <c r="E3" s="12" t="s">
         <v>6</v>
       </c>
-      <c r="F3" s="9"/>
+      <c r="F3" s="7"/>
     </row>
     <row r="4" spans="2:6">
-      <c r="B4" s="12"/>
-      <c r="C4" s="13"/>
-      <c r="D4" s="14" t="b">
+      <c r="B4" s="10"/>
+      <c r="C4" s="11"/>
+      <c r="D4" s="12" t="b">
         <v>0</v>
       </c>
-      <c r="E4" s="14" t="s">
+      <c r="E4" s="12" t="s">
         <v>7</v>
       </c>
-      <c r="F4" s="9"/>
+      <c r="F4" s="7"/>
     </row>
     <row r="5" spans="2:6">
-      <c r="B5" s="12"/>
-      <c r="C5" s="15" t="s">
+      <c r="B5" s="10"/>
+      <c r="C5" s="11" t="s">
         <v>8</v>
       </c>
-      <c r="D5" s="14" t="b">
+      <c r="D5" s="12" t="b">
         <v>1</v>
       </c>
-      <c r="E5" s="14" t="s">
+      <c r="E5" s="12" t="s">
         <v>9</v>
       </c>
-      <c r="F5" s="9"/>
+      <c r="F5" s="7"/>
     </row>
     <row r="6" spans="2:6">
-      <c r="B6" s="12"/>
-      <c r="C6" s="15"/>
-      <c r="D6" s="14" t="b">
+      <c r="B6" s="10"/>
+      <c r="C6" s="11"/>
+      <c r="D6" s="12" t="b">
         <v>0</v>
       </c>
-      <c r="E6" s="14" t="s">
+      <c r="E6" s="12" t="s">
         <v>10</v>
       </c>
-      <c r="F6" s="9"/>
+      <c r="F6" s="7"/>
     </row>
     <row r="7" spans="2:6">
-      <c r="B7" s="12"/>
-      <c r="C7" s="15" t="s">
+      <c r="B7" s="10"/>
+      <c r="C7" s="11" t="s">
         <v>11</v>
       </c>
-      <c r="D7" s="14" t="b">
+      <c r="D7" s="12" t="b">
         <v>1</v>
       </c>
-      <c r="E7" s="14" t="s">
+      <c r="E7" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="F7" s="9"/>
+      <c r="F7" s="7"/>
     </row>
     <row r="8" spans="2:6">
-      <c r="B8" s="12"/>
-      <c r="C8" s="15"/>
-      <c r="D8" s="14" t="b">
+      <c r="B8" s="10"/>
+      <c r="C8" s="11"/>
+      <c r="D8" s="12" t="b">
         <v>0</v>
       </c>
-      <c r="E8" s="14" t="s">
+      <c r="E8" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="F8" s="9"/>
+      <c r="F8" s="7"/>
     </row>
     <row r="9" spans="2:6">
-      <c r="B9" s="12"/>
-      <c r="C9" s="13" t="s">
+      <c r="B9" s="10"/>
+      <c r="C9" s="11" t="s">
         <v>14</v>
       </c>
-      <c r="D9" s="14" t="b">
+      <c r="D9" s="12" t="b">
         <v>1</v>
       </c>
-      <c r="E9" s="14" t="s">
+      <c r="E9" s="12" t="s">
         <v>15</v>
       </c>
-      <c r="F9" s="9"/>
+      <c r="F9" s="7"/>
     </row>
     <row r="10" spans="2:6">
-      <c r="B10" s="12"/>
-      <c r="C10" s="13"/>
-      <c r="D10" s="14" t="b">
+      <c r="B10" s="10"/>
+      <c r="C10" s="11"/>
+      <c r="D10" s="12" t="b">
         <v>0</v>
       </c>
-      <c r="E10" s="14" t="s">
+      <c r="E10" s="12" t="s">
         <v>16</v>
       </c>
-      <c r="F10" s="9"/>
+      <c r="F10" s="7"/>
     </row>
     <row r="11" spans="2:6">
-      <c r="B11" s="12" t="s">
+      <c r="B11" s="10" t="s">
         <v>17</v>
       </c>
-      <c r="C11" s="16" t="s">
+      <c r="C11" s="13" t="s">
         <v>18</v>
       </c>
-      <c r="D11" s="14" t="b">
+      <c r="D11" s="12" t="b">
         <v>1</v>
       </c>
-      <c r="E11" s="14" t="s">
+      <c r="E11" s="12" t="s">
         <v>19</v>
       </c>
-      <c r="F11" s="9"/>
+      <c r="F11" s="7"/>
     </row>
     <row r="12" spans="2:6">
-      <c r="B12" s="12"/>
-      <c r="C12" s="16"/>
-      <c r="D12" s="14" t="b">
+      <c r="B12" s="10"/>
+      <c r="C12" s="13"/>
+      <c r="D12" s="12" t="b">
         <v>0</v>
       </c>
-      <c r="E12" s="14" t="s">
+      <c r="E12" s="12" t="s">
         <v>20</v>
       </c>
-      <c r="F12" s="9"/>
+      <c r="F12" s="7"/>
     </row>
     <row r="13" spans="2:6">
-      <c r="B13" s="12"/>
-      <c r="C13" s="16" t="s">
+      <c r="B13" s="10"/>
+      <c r="C13" s="13" t="s">
         <v>21</v>
       </c>
-      <c r="D13" s="14" t="b">
+      <c r="D13" s="12" t="b">
         <v>1</v>
       </c>
-      <c r="E13" s="14" t="s">
+      <c r="E13" s="12" t="s">
         <v>22</v>
       </c>
-      <c r="F13" s="9"/>
+      <c r="F13" s="7"/>
     </row>
     <row r="14" spans="2:5">
-      <c r="B14" s="12"/>
-      <c r="C14" s="16"/>
-      <c r="D14" s="14" t="b">
+      <c r="B14" s="10"/>
+      <c r="C14" s="13"/>
+      <c r="D14" s="12" t="b">
         <v>0</v>
       </c>
-      <c r="E14" s="14" t="s">
+      <c r="E14" s="12" t="s">
         <v>23</v>
       </c>
     </row>
@@ -2075,36 +2095,36 @@
       <c r="C4" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="D4" s="4"/>
+      <c r="D4" s="3"/>
     </row>
     <row r="5" spans="2:4">
-      <c r="B5" s="5"/>
-      <c r="C5" s="6" t="b">
+      <c r="B5" s="4"/>
+      <c r="C5" s="5" t="b">
         <v>1</v>
       </c>
-      <c r="D5" s="6" t="b">
+      <c r="D5" s="5" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="6" ht="57.6" spans="2:4">
-      <c r="B6" s="7" t="b">
+      <c r="B6" s="4" t="b">
         <v>1</v>
       </c>
-      <c r="C6" s="17" t="s">
+      <c r="C6" s="14" t="s">
         <v>25</v>
       </c>
-      <c r="D6" s="17" t="s">
+      <c r="D6" s="14" t="s">
         <v>26</v>
       </c>
     </row>
     <row r="7" ht="72" spans="2:4">
-      <c r="B7" s="7" t="b">
+      <c r="B7" s="4" t="b">
         <v>0</v>
       </c>
-      <c r="C7" s="17" t="s">
+      <c r="C7" s="14" t="s">
         <v>27</v>
       </c>
-      <c r="D7" s="17" t="s">
+      <c r="D7" s="14" t="s">
         <v>28</v>
       </c>
     </row>
@@ -2120,36 +2140,36 @@
       <c r="C12" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="D12" s="4"/>
+      <c r="D12" s="3"/>
     </row>
     <row r="13" spans="2:4">
-      <c r="B13" s="5"/>
-      <c r="C13" s="6" t="b">
+      <c r="B13" s="4"/>
+      <c r="C13" s="5" t="b">
         <v>1</v>
       </c>
-      <c r="D13" s="6" t="b">
+      <c r="D13" s="5" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="14" spans="2:4">
-      <c r="B14" s="7" t="b">
+      <c r="B14" s="4" t="b">
         <v>1</v>
       </c>
-      <c r="C14" s="8" t="s">
+      <c r="C14" s="6" t="s">
         <v>30</v>
       </c>
-      <c r="D14" s="8" t="s">
+      <c r="D14" s="6" t="s">
         <v>31</v>
       </c>
     </row>
     <row r="15" spans="2:4">
-      <c r="B15" s="7" t="b">
+      <c r="B15" s="4" t="b">
         <v>0</v>
       </c>
-      <c r="C15" s="8" t="s">
+      <c r="C15" s="6" t="s">
         <v>30</v>
       </c>
-      <c r="D15" s="8" t="s">
+      <c r="D15" s="6" t="s">
         <v>32</v>
       </c>
     </row>

</xml_diff>